<commit_message>
feat: Verify existed files
</commit_message>
<xml_diff>
--- a/__chapter-2/hw2/menu/report-electricity-bill.xlsx
+++ b/__chapter-2/hw2/menu/report-electricity-bill.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,7 +444,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>loitpg</t>
+          <t>loiasd</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -452,6 +452,22 @@
       </c>
       <c r="D2" t="n">
         <v>665000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>aosdij</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>250</v>
+      </c>
+      <c r="D3" t="n">
+        <v>590000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>